<commit_message>
feat: change Aisha Joosub's code from AISHA10 to FOUNDER10
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/influencer-affiliate-links.xlsx
+++ b/influencer-affiliate-links.xlsx
@@ -2429,10 +2429,10 @@
         <v>Joosub</v>
       </c>
       <c r="E64" t="str">
-        <v>AISHA10</v>
+        <v>FOUNDER10</v>
       </c>
       <c r="F64" t="str">
-        <v>https://www.ayooshonline.com/products?ref=AISHA10</v>
+        <v>https://www.ayooshonline.com/products?ref=FOUNDER10</v>
       </c>
       <c r="G64" t="str">
         <v>5%</v>
@@ -2444,7 +2444,7 @@
         <v>24/07/2026</v>
       </c>
       <c r="J64" t="str">
-        <v>AISHA10</v>
+        <v>FOUNDER10</v>
       </c>
     </row>
     <row r="65">

</xml_diff>